<commit_message>
update main board schematic
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayde\hackclubprojects\SRAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE860CC-F034-4478-94AF-93851B3D18B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5734E93-95FD-44B2-A576-804991C59D42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{34E5001A-E530-4D7D-A47C-599746382A99}"/>
+    <workbookView xWindow="6435" yWindow="5430" windowWidth="21600" windowHeight="12645" xr2:uid="{34E5001A-E530-4D7D-A47C-599746382A99}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -303,16 +303,16 @@
     <t>GRAND TOTAL</t>
   </si>
   <si>
-    <t>https://www.lcsc.com/product-detail/C77101.html</t>
-  </si>
-  <si>
-    <t>muRata GRM32ER61C476KE15L</t>
-  </si>
-  <si>
     <t>https://www.lcsc.com/product-detail/C7461243.html</t>
   </si>
   <si>
     <t>KNSCHA 126RV0112</t>
+  </si>
+  <si>
+    <t>HRE CGA1206X5R476M250NT</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C6119973.html</t>
   </si>
 </sst>
 </file>
@@ -911,19 +911,19 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B12" s="8">
         <v>10</v>
       </c>
       <c r="C12" s="9">
-        <v>3.14</v>
+        <v>2.88</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>26</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -1149,7 +1149,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B30" s="15">
         <v>40</v>
@@ -1161,7 +1161,7 @@
         <v>67</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="C39" s="1">
         <f>SUM(C2:C38)</f>
-        <v>754.59999999999991</v>
+        <v>754.33999999999992</v>
       </c>
     </row>
   </sheetData>
@@ -1250,21 +1250,21 @@
     <hyperlink ref="E9" r:id="rId5" xr:uid="{AF1D5E71-8A26-4861-AB6C-BA5B73B558B5}"/>
     <hyperlink ref="E11" r:id="rId6" xr:uid="{EAA0FE3F-4210-4197-8A84-3E311B1E0DD4}"/>
     <hyperlink ref="E10" r:id="rId7" xr:uid="{E6B30901-51DC-48D1-A00D-9CC15A311090}"/>
-    <hyperlink ref="E12" r:id="rId8" xr:uid="{55E9EF0E-35D6-4789-80A5-B868EF71F9E3}"/>
-    <hyperlink ref="E13" r:id="rId9" xr:uid="{655DD5A6-3680-402D-A213-E373ED0A04B3}"/>
-    <hyperlink ref="E14" r:id="rId10" xr:uid="{E6DF9F36-757E-4476-BD70-28F7E1F99F70}"/>
-    <hyperlink ref="E15" r:id="rId11" xr:uid="{1AC84DE5-6CCA-42CC-80AC-70114945119B}"/>
-    <hyperlink ref="E16" r:id="rId12" xr:uid="{69CEFA70-F3C1-42F1-B023-1EA7E7A16646}"/>
-    <hyperlink ref="E17" r:id="rId13" xr:uid="{F23FE842-6DB6-4E4F-A145-C3FAB5F46BB5}"/>
-    <hyperlink ref="E18" r:id="rId14" xr:uid="{96D480BA-3143-4D27-910A-8DB63BD9911E}"/>
-    <hyperlink ref="E19" r:id="rId15" xr:uid="{FC1E44E0-E492-40A7-BA72-858E311F0E6B}"/>
-    <hyperlink ref="E20" r:id="rId16" xr:uid="{8FCF208D-DB1E-4B78-8F0B-0862090DF17C}"/>
-    <hyperlink ref="E21" r:id="rId17" xr:uid="{4D2E9F39-BBF0-4ED5-A3F4-155FDCE0EE23}"/>
-    <hyperlink ref="E22" r:id="rId18" xr:uid="{2A107639-C50E-4692-BCD5-0196CE4739AB}"/>
-    <hyperlink ref="E4" r:id="rId19" xr:uid="{844DA8A5-FB35-4F0B-A1F4-8116A748C40E}"/>
-    <hyperlink ref="E31" r:id="rId20" xr:uid="{5600F95F-40E7-4F55-A313-2023A5F400B9}"/>
-    <hyperlink ref="E32" r:id="rId21" xr:uid="{9D311E0B-996E-4B99-B32A-9F25E8B76079}"/>
-    <hyperlink ref="E30" r:id="rId22" xr:uid="{603F2D51-63FE-4820-93B9-30767E19C3CC}"/>
+    <hyperlink ref="E13" r:id="rId8" xr:uid="{655DD5A6-3680-402D-A213-E373ED0A04B3}"/>
+    <hyperlink ref="E14" r:id="rId9" xr:uid="{E6DF9F36-757E-4476-BD70-28F7E1F99F70}"/>
+    <hyperlink ref="E15" r:id="rId10" xr:uid="{1AC84DE5-6CCA-42CC-80AC-70114945119B}"/>
+    <hyperlink ref="E16" r:id="rId11" xr:uid="{69CEFA70-F3C1-42F1-B023-1EA7E7A16646}"/>
+    <hyperlink ref="E17" r:id="rId12" xr:uid="{F23FE842-6DB6-4E4F-A145-C3FAB5F46BB5}"/>
+    <hyperlink ref="E18" r:id="rId13" xr:uid="{96D480BA-3143-4D27-910A-8DB63BD9911E}"/>
+    <hyperlink ref="E19" r:id="rId14" xr:uid="{FC1E44E0-E492-40A7-BA72-858E311F0E6B}"/>
+    <hyperlink ref="E20" r:id="rId15" xr:uid="{8FCF208D-DB1E-4B78-8F0B-0862090DF17C}"/>
+    <hyperlink ref="E21" r:id="rId16" xr:uid="{4D2E9F39-BBF0-4ED5-A3F4-155FDCE0EE23}"/>
+    <hyperlink ref="E22" r:id="rId17" xr:uid="{2A107639-C50E-4692-BCD5-0196CE4739AB}"/>
+    <hyperlink ref="E4" r:id="rId18" xr:uid="{844DA8A5-FB35-4F0B-A1F4-8116A748C40E}"/>
+    <hyperlink ref="E31" r:id="rId19" xr:uid="{5600F95F-40E7-4F55-A313-2023A5F400B9}"/>
+    <hyperlink ref="E32" r:id="rId20" xr:uid="{9D311E0B-996E-4B99-B32A-9F25E8B76079}"/>
+    <hyperlink ref="E30" r:id="rId21" xr:uid="{603F2D51-63FE-4820-93B9-30767E19C3CC}"/>
+    <hyperlink ref="E12" r:id="rId22" xr:uid="{28A0EBB7-2304-492C-A951-78F5F394482B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId23"/>

</xml_diff>

<commit_message>
Add breakout board through holes on main ram board
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayde\hackclubprojects\SRAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1BD4F1D-3F24-4CA1-BAF6-EB06480ED52E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F907423-6D94-4BCD-88DA-FF38C8CFDAAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="2415" windowWidth="21600" windowHeight="12645" xr2:uid="{34E5001A-E530-4D7D-A47C-599746382A99}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{34E5001A-E530-4D7D-A47C-599746382A99}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="88">
   <si>
     <t>Item</t>
   </si>
@@ -264,24 +264,9 @@
     <t>some more capacitors (100u)</t>
   </si>
   <si>
-    <t>Yongyu Photoelectric SZYY0805R</t>
-  </si>
-  <si>
     <t>red leds</t>
   </si>
   <si>
-    <t>https://www.lcsc.com/product-detail/C434431.html</t>
-  </si>
-  <si>
-    <t>FOJAN FRC0805F2200TS</t>
-  </si>
-  <si>
-    <t>resistors (220) for led circuit</t>
-  </si>
-  <si>
-    <t>https://www.lcsc.com/product-detail/C2933369.html</t>
-  </si>
-  <si>
     <t xml:space="preserve">JLCPCB shipping + tarrifs </t>
   </si>
   <si>
@@ -322,6 +307,30 @@
   </si>
   <si>
     <t>including the mosfets and some misc for it</t>
+  </si>
+  <si>
+    <t>Yongyu PhotXINGLIGHT XL-2012SURC-FJoelectric SZYY0805R</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C7371909.html</t>
+  </si>
+  <si>
+    <t>resistors (360) for led circuit</t>
+  </si>
+  <si>
+    <t>FOJAN FRC0805F3600TS</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C2930158.html</t>
+  </si>
+  <si>
+    <t>hanxia HX PZ1.0-1x2P ZZ</t>
+  </si>
+  <si>
+    <t>pin headers, small</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C22438170.html</t>
   </si>
 </sst>
 </file>
@@ -754,7 +763,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED1153EB-BB1E-4BE6-92B6-2B30F9AD7E28}">
-  <dimension ref="A1:F40"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.5703125" customWidth="1"/>
@@ -903,7 +912,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B11" s="8">
         <v>20</v>
@@ -915,12 +924,12 @@
         <v>21</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B12" s="8">
         <v>10</v>
@@ -932,7 +941,7 @@
         <v>24</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -954,7 +963,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B14" s="8">
         <v>100</v>
@@ -963,10 +972,10 @@
         <v>0.35</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1167,7 +1176,7 @@
         <v>400</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E30" s="14" t="s">
         <v>59</v>
@@ -1175,7 +1184,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B31" s="15">
         <v>100</v>
@@ -1187,29 +1196,29 @@
         <v>64</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="14" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B32" s="15">
         <v>500</v>
       </c>
       <c r="C32" s="16">
-        <v>5.8</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>67</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="B33" s="15">
         <v>500</v>
@@ -1218,53 +1227,70 @@
         <v>1.6</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C36" s="5">
-        <v>100</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>59</v>
+        <v>84</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B34" s="2">
+        <v>150</v>
+      </c>
+      <c r="C34" s="1">
+        <v>4.8600000000000003</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="E34" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>59</v>
       </c>
       <c r="C37" s="5">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E37" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>74</v>
-      </c>
-      <c r="C40" s="1">
-        <f>SUM(C2:C39)</f>
-        <v>763.82999999999993</v>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C38" s="5">
+        <v>50</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>69</v>
+      </c>
+      <c r="C41" s="1">
+        <f>SUM(C2:C40)</f>
+        <v>771.68999999999994</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
create schematic for input board and footprints
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayde\hackclubprojects\SRAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F907423-6D94-4BCD-88DA-FF38C8CFDAAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD0312AA-4CDA-4F35-B263-00E71DFC79E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{34E5001A-E530-4D7D-A47C-599746382A99}"/>
   </bookViews>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="93">
   <si>
     <t>Item</t>
   </si>
@@ -331,6 +331,21 @@
   </si>
   <si>
     <t>https://www.lcsc.com/product-detail/C22438170.html</t>
+  </si>
+  <si>
+    <t>SHOU HAN TS6665CJ 250gf 009</t>
+  </si>
+  <si>
+    <t>push buttons</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C5359346.html</t>
+  </si>
+  <si>
+    <t>PCB (input board)</t>
+  </si>
+  <si>
+    <t>pcb</t>
   </si>
 </sst>
 </file>
@@ -364,7 +379,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -395,6 +410,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFF5B"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -409,7 +430,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -428,6 +449,10 @@
     <xf numFmtId="1" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -435,6 +460,12 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFDCFF5B"/>
+      <color rgb="FFFFB9B9"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -763,7 +794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED1153EB-BB1E-4BE6-92B6-2B30F9AD7E28}">
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.5703125" customWidth="1"/>
@@ -1251,46 +1282,80 @@
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
+      <c r="A37" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="B37" s="19">
+        <v>150</v>
+      </c>
+      <c r="C37" s="20">
+        <v>2.31</v>
+      </c>
+      <c r="D37" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="E37" s="21" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="B38" s="19">
+        <v>1</v>
+      </c>
+      <c r="C38" s="20">
+        <v>15</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B37" s="4" t="s">
+      <c r="B41" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C41" s="5">
         <v>100</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D41" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="E41" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B42" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C38" s="5">
+      <c r="C42" s="5">
         <v>50</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D42" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E38" s="3" t="s">
+      <c r="E42" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>69</v>
       </c>
-      <c r="C41" s="1">
-        <f>SUM(C2:C40)</f>
-        <v>771.68999999999994</v>
+      <c r="C45" s="1">
+        <f>SUM(C2:C44)</f>
+        <v>788.99999999999989</v>
       </c>
     </row>
   </sheetData>
@@ -1318,8 +1383,9 @@
     <hyperlink ref="E31" r:id="rId21" xr:uid="{603F2D51-63FE-4820-93B9-30767E19C3CC}"/>
     <hyperlink ref="E12" r:id="rId22" xr:uid="{28A0EBB7-2304-492C-A951-78F5F394482B}"/>
     <hyperlink ref="E14" r:id="rId23" xr:uid="{6ED20A36-8F40-483A-BE25-4C87A2D92BFB}"/>
+    <hyperlink ref="E37" r:id="rId24" xr:uid="{658E5E28-83C4-44FC-A8A9-EE933E75693B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId24"/>
+  <legacyDrawing r:id="rId25"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
finish main input board
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayde\hackclubprojects\SRAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD0312AA-4CDA-4F35-B263-00E71DFC79E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FAEF2B5-344D-41C4-9ECB-AFE1882AA118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{34E5001A-E530-4D7D-A47C-599746382A99}"/>
   </bookViews>
@@ -315,37 +315,37 @@
     <t>https://www.lcsc.com/product-detail/C7371909.html</t>
   </si>
   <si>
-    <t>resistors (360) for led circuit</t>
-  </si>
-  <si>
-    <t>FOJAN FRC0805F3600TS</t>
-  </si>
-  <si>
-    <t>https://www.lcsc.com/product-detail/C2930158.html</t>
-  </si>
-  <si>
     <t>hanxia HX PZ1.0-1x2P ZZ</t>
   </si>
   <si>
     <t>pin headers, small</t>
   </si>
   <si>
-    <t>https://www.lcsc.com/product-detail/C22438170.html</t>
-  </si>
-  <si>
-    <t>SHOU HAN TS6665CJ 250gf 009</t>
-  </si>
-  <si>
     <t>push buttons</t>
   </si>
   <si>
-    <t>https://www.lcsc.com/product-detail/C5359346.html</t>
-  </si>
-  <si>
     <t>PCB (input board)</t>
   </si>
   <si>
     <t>pcb</t>
+  </si>
+  <si>
+    <t>resistors (180) for led circuit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C22438170.html </t>
+  </si>
+  <si>
+    <t>FOJAN FRC0805F1800TS</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C2933344.html</t>
+  </si>
+  <si>
+    <t>SHOU HAN TS4538TP 250gf 009</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C5359325.html</t>
   </si>
 </sst>
 </file>
@@ -430,7 +430,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -453,6 +453,7 @@
     <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1249,24 +1250,24 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="B33" s="15">
         <v>500</v>
       </c>
       <c r="C33" s="16">
-        <v>1.6</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B34" s="2">
         <v>150</v>
@@ -1275,32 +1276,32 @@
         <v>4.8600000000000003</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="E34" t="s">
-        <v>87</v>
+        <v>83</v>
+      </c>
+      <c r="E34" s="22" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B37" s="19">
         <v>150</v>
       </c>
       <c r="C37" s="20">
-        <v>2.31</v>
+        <v>2.61</v>
       </c>
       <c r="D37" s="18" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B38" s="19">
         <v>1</v>
@@ -1309,7 +1310,7 @@
         <v>15</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E38" s="18" t="s">
         <v>59</v>
@@ -1355,7 +1356,7 @@
       </c>
       <c r="C45" s="1">
         <f>SUM(C2:C44)</f>
-        <v>788.99999999999989</v>
+        <v>788.84999999999991</v>
       </c>
     </row>
   </sheetData>
@@ -1384,8 +1385,9 @@
     <hyperlink ref="E12" r:id="rId22" xr:uid="{28A0EBB7-2304-492C-A951-78F5F394482B}"/>
     <hyperlink ref="E14" r:id="rId23" xr:uid="{6ED20A36-8F40-483A-BE25-4C87A2D92BFB}"/>
     <hyperlink ref="E37" r:id="rId24" xr:uid="{658E5E28-83C4-44FC-A8A9-EE933E75693B}"/>
+    <hyperlink ref="E34" r:id="rId25" xr:uid="{6F005684-77F1-49B6-9BD6-CB4A7DAA5FC5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId25"/>
+  <legacyDrawing r:id="rId26"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update bom, add more capacitors
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jayde\hackclubprojects\SRAM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FAEF2B5-344D-41C4-9ECB-AFE1882AA118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B05134-CCDC-4B21-AF8B-590207369480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{34E5001A-E530-4D7D-A47C-599746382A99}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{34E5001A-E530-4D7D-A47C-599746382A99}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,8 @@
 Orange: for multiple boards
 Green: for main controller board
 Blue: for main demux board
-Purple: for the ram boards</t>
+Purple: for the ram boards
+Yellow-green: for the input board</t>
         </r>
       </text>
     </comment>
@@ -67,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="102">
   <si>
     <t>Item</t>
   </si>
@@ -84,24 +85,12 @@
     <t>URL</t>
   </si>
   <si>
-    <t>JTD JTD2302B</t>
-  </si>
-  <si>
     <t>n-mosfets</t>
   </si>
   <si>
-    <t>https://www.lcsc.com/product-detail/C49308282.html</t>
-  </si>
-  <si>
-    <t>DOINGTER DO2301E-Q</t>
-  </si>
-  <si>
     <t>p-mosfets</t>
   </si>
   <si>
-    <t>https://www.lcsc.com/product-detail/C41384537.html</t>
-  </si>
-  <si>
     <t>https://www.lcsc.com/product-detail/C3039987.html</t>
   </si>
   <si>
@@ -306,9 +295,6 @@
     <t>https://www.lcsc.com/product-detail/C115323.html</t>
   </si>
   <si>
-    <t>including the mosfets and some misc for it</t>
-  </si>
-  <si>
     <t>Yongyu PhotXINGLIGHT XL-2012SURC-FJoelectric SZYY0805R</t>
   </si>
   <si>
@@ -346,6 +332,48 @@
   </si>
   <si>
     <t>https://www.lcsc.com/product-detail/C5359325.html</t>
+  </si>
+  <si>
+    <t>OSEN 2300</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C20607736.html</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C20607737.html</t>
+  </si>
+  <si>
+    <t>OSEN 2301</t>
+  </si>
+  <si>
+    <t>including the 20 thousand mosfets</t>
+  </si>
+  <si>
+    <t>RS-03K47R0FT</t>
+  </si>
+  <si>
+    <t>included in pcb price, 47 ohm resistors</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C140087.html</t>
+  </si>
+  <si>
+    <t>FOJAN FRC0603F1002TS</t>
+  </si>
+  <si>
+    <t>included in pcb price, 10k ohm resistors</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C2906982.html</t>
+  </si>
+  <si>
+    <t>Lian Xin Technology XDFH-0254-2*20P</t>
+  </si>
+  <si>
+    <t>idc headers, right angle</t>
+  </si>
+  <si>
+    <t>https://www.lcsc.com/product-detail/C19193815.html</t>
   </si>
 </sst>
 </file>
@@ -430,7 +458,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -453,7 +481,6 @@
     <xf numFmtId="1" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -795,7 +822,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED1153EB-BB1E-4BE6-92B6-2B30F9AD7E28}">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.5703125" customWidth="1"/>
@@ -825,245 +852,245 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>5</v>
+        <v>88</v>
       </c>
       <c r="B2" s="4">
         <v>3000</v>
       </c>
       <c r="C2" s="5">
-        <v>27</v>
+        <v>16.8</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>7</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>8</v>
+        <v>91</v>
       </c>
       <c r="B3" s="4">
         <v>3000</v>
       </c>
       <c r="C3" s="5">
-        <v>26.7</v>
+        <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>10</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B4" s="4">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C4" s="5">
-        <v>21.55</v>
+        <v>15.32</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="8">
-        <v>15</v>
-      </c>
-      <c r="C7" s="9">
-        <v>6.35</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>11</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" s="4">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5">
+        <v>8.7200000000000006</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B8" s="8">
+        <v>15</v>
+      </c>
+      <c r="C8" s="9">
+        <v>6.35</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="8">
         <v>50</v>
       </c>
-      <c r="C8" s="9">
+      <c r="C9" s="9">
         <v>0.43</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="4">
-        <v>600</v>
-      </c>
-      <c r="C9" s="5">
-        <v>7.68</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>18</v>
+      <c r="D9" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="4">
+        <v>600</v>
+      </c>
+      <c r="C10" s="5">
+        <v>7.68</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="4">
+      <c r="E10" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="4">
         <v>500</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C11" s="5">
         <v>4.4000000000000004</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="8">
-        <v>20</v>
-      </c>
-      <c r="C11" s="9">
-        <v>0.78</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" s="10" t="s">
-        <v>75</v>
+      <c r="D11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B12" s="8">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C12" s="9">
-        <v>2.88</v>
+        <v>0.78</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="B13" s="8">
         <v>10</v>
       </c>
       <c r="C13" s="9">
-        <v>2.5299999999999998</v>
+        <v>2.88</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>27</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>76</v>
+        <v>21</v>
       </c>
       <c r="B14" s="8">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C14" s="9">
-        <v>0.35</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>78</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="B15" s="8">
         <v>100</v>
       </c>
       <c r="C15" s="9">
-        <v>0.42</v>
+        <v>0.35</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>29</v>
+        <v>73</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>30</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="B16" s="8">
         <v>100</v>
       </c>
       <c r="C16" s="9">
-        <v>0.41</v>
+        <v>0.42</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B17" s="8">
         <v>100</v>
       </c>
       <c r="C17" s="9">
-        <v>0.32</v>
+        <v>0.41</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B18" s="8">
         <v>100</v>
@@ -1072,15 +1099,15 @@
         <v>0.32</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B19" s="8">
         <v>100</v>
@@ -1089,305 +1116,359 @@
         <v>0.32</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="B20" s="8">
         <v>100</v>
       </c>
       <c r="C20" s="9">
+        <v>0.32</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="8">
+        <v>100</v>
+      </c>
+      <c r="C21" s="9">
         <v>0.3</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D21" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="4">
+        <v>100</v>
+      </c>
+      <c r="C22" s="5">
+        <v>0.27</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B21" s="4">
-        <v>100</v>
-      </c>
-      <c r="C21" s="5">
-        <v>0.27</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B22" s="8">
-        <v>100</v>
-      </c>
-      <c r="C22" s="9">
-        <v>0.32</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="B23" s="8">
         <v>100</v>
       </c>
       <c r="C23" s="9">
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="B24" s="8">
+        <v>100</v>
+      </c>
+      <c r="C24" s="9">
+        <v>0.33</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E24" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" s="8">
         <v>1</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C25" s="9">
         <v>50</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D25" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="12">
+        <v>1</v>
+      </c>
+      <c r="C28" s="13">
+        <v>48.37</v>
+      </c>
+      <c r="D28" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="E24" s="7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" s="12">
-        <v>1</v>
-      </c>
-      <c r="C27" s="13">
-        <v>48.37</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>62</v>
-      </c>
-      <c r="E27" s="11" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="B30" s="15">
-        <v>16</v>
-      </c>
-      <c r="C30" s="16">
-        <v>400</v>
-      </c>
-      <c r="D30" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>59</v>
+      <c r="E28" s="11" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="B31" s="15">
+        <v>17</v>
+      </c>
+      <c r="C31" s="16">
+        <v>380</v>
+      </c>
+      <c r="D31" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B32" s="4">
         <v>100</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C32" s="5">
         <v>4.4000000000000004</v>
       </c>
-      <c r="D31" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="E31" s="17" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B32" s="15">
-        <v>500</v>
-      </c>
-      <c r="C32" s="16">
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="D32" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E32" s="17" t="s">
-        <v>81</v>
+      <c r="D32" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="B33" s="15">
         <v>500</v>
       </c>
       <c r="C33" s="16">
-        <v>1.1499999999999999</v>
+        <v>8.8000000000000007</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B34" s="15">
+        <v>500</v>
+      </c>
+      <c r="C34" s="16">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="D34" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="B34" s="2">
+      <c r="E34" s="17" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" s="15">
         <v>150</v>
       </c>
-      <c r="C34" s="1">
+      <c r="C35" s="16">
         <v>4.8600000000000003</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="D35" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="E35" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="E34" s="22" t="s">
-        <v>88</v>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B36" s="15">
+        <v>2186</v>
+      </c>
+      <c r="C36" s="16">
+        <v>0</v>
+      </c>
+      <c r="D36" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="18" t="s">
-        <v>91</v>
-      </c>
-      <c r="B37" s="19">
+      <c r="A37" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B37" s="15">
+        <v>282</v>
+      </c>
+      <c r="C37" s="16">
+        <v>0</v>
+      </c>
+      <c r="D37" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B40" s="19">
         <v>150</v>
       </c>
-      <c r="C37" s="20">
+      <c r="C40" s="20">
         <v>2.61</v>
       </c>
-      <c r="D37" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="E37" s="21" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="B38" s="19">
+      <c r="D40" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" s="21" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="B41" s="19">
         <v>1</v>
       </c>
-      <c r="C38" s="20">
+      <c r="C41" s="20">
         <v>15</v>
       </c>
-      <c r="D38" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="E38" s="18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C41" s="5">
+      <c r="D41" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="E41" s="18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C44" s="5">
         <v>100</v>
       </c>
-      <c r="D41" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E41" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C42" s="5">
+      <c r="D44" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" s="5">
         <v>50</v>
       </c>
-      <c r="D42" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>69</v>
-      </c>
-      <c r="C45" s="1">
-        <f>SUM(C2:C44)</f>
-        <v>788.84999999999991</v>
+      <c r="D45" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E45" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>65</v>
+      </c>
+      <c r="C48" s="1">
+        <f>SUM(C2:C47)</f>
+        <v>755.43999999999994</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="E8" r:id="rId1" xr:uid="{15215B3D-FA5E-48FB-8EE7-EB176E394B70}"/>
-    <hyperlink ref="E7" r:id="rId2" xr:uid="{98CCC44D-DB76-4EE9-94CF-F37FAEA9BCB5}"/>
+    <hyperlink ref="E9" r:id="rId1" xr:uid="{15215B3D-FA5E-48FB-8EE7-EB176E394B70}"/>
+    <hyperlink ref="E8" r:id="rId2" xr:uid="{98CCC44D-DB76-4EE9-94CF-F37FAEA9BCB5}"/>
     <hyperlink ref="E3" r:id="rId3" xr:uid="{D9E20DA9-C275-4CE9-AF20-9AEF60D976F5}"/>
     <hyperlink ref="E2" r:id="rId4" xr:uid="{2677350B-8551-4DBC-A88A-2FE3589255E8}"/>
-    <hyperlink ref="E9" r:id="rId5" xr:uid="{AF1D5E71-8A26-4861-AB6C-BA5B73B558B5}"/>
-    <hyperlink ref="E11" r:id="rId6" xr:uid="{EAA0FE3F-4210-4197-8A84-3E311B1E0DD4}"/>
-    <hyperlink ref="E10" r:id="rId7" xr:uid="{E6B30901-51DC-48D1-A00D-9CC15A311090}"/>
-    <hyperlink ref="E13" r:id="rId8" xr:uid="{655DD5A6-3680-402D-A213-E373ED0A04B3}"/>
-    <hyperlink ref="E15" r:id="rId9" xr:uid="{E6DF9F36-757E-4476-BD70-28F7E1F99F70}"/>
-    <hyperlink ref="E16" r:id="rId10" xr:uid="{1AC84DE5-6CCA-42CC-80AC-70114945119B}"/>
-    <hyperlink ref="E17" r:id="rId11" xr:uid="{69CEFA70-F3C1-42F1-B023-1EA7E7A16646}"/>
-    <hyperlink ref="E18" r:id="rId12" xr:uid="{F23FE842-6DB6-4E4F-A145-C3FAB5F46BB5}"/>
-    <hyperlink ref="E19" r:id="rId13" xr:uid="{96D480BA-3143-4D27-910A-8DB63BD9911E}"/>
-    <hyperlink ref="E20" r:id="rId14" xr:uid="{FC1E44E0-E492-40A7-BA72-858E311F0E6B}"/>
-    <hyperlink ref="E21" r:id="rId15" xr:uid="{8FCF208D-DB1E-4B78-8F0B-0862090DF17C}"/>
-    <hyperlink ref="E22" r:id="rId16" xr:uid="{4D2E9F39-BBF0-4ED5-A3F4-155FDCE0EE23}"/>
-    <hyperlink ref="E23" r:id="rId17" xr:uid="{2A107639-C50E-4692-BCD5-0196CE4739AB}"/>
+    <hyperlink ref="E10" r:id="rId5" xr:uid="{AF1D5E71-8A26-4861-AB6C-BA5B73B558B5}"/>
+    <hyperlink ref="E12" r:id="rId6" xr:uid="{EAA0FE3F-4210-4197-8A84-3E311B1E0DD4}"/>
+    <hyperlink ref="E11" r:id="rId7" xr:uid="{E6B30901-51DC-48D1-A00D-9CC15A311090}"/>
+    <hyperlink ref="E14" r:id="rId8" xr:uid="{655DD5A6-3680-402D-A213-E373ED0A04B3}"/>
+    <hyperlink ref="E16" r:id="rId9" xr:uid="{E6DF9F36-757E-4476-BD70-28F7E1F99F70}"/>
+    <hyperlink ref="E17" r:id="rId10" xr:uid="{1AC84DE5-6CCA-42CC-80AC-70114945119B}"/>
+    <hyperlink ref="E18" r:id="rId11" xr:uid="{69CEFA70-F3C1-42F1-B023-1EA7E7A16646}"/>
+    <hyperlink ref="E19" r:id="rId12" xr:uid="{F23FE842-6DB6-4E4F-A145-C3FAB5F46BB5}"/>
+    <hyperlink ref="E20" r:id="rId13" xr:uid="{96D480BA-3143-4D27-910A-8DB63BD9911E}"/>
+    <hyperlink ref="E21" r:id="rId14" xr:uid="{FC1E44E0-E492-40A7-BA72-858E311F0E6B}"/>
+    <hyperlink ref="E22" r:id="rId15" xr:uid="{8FCF208D-DB1E-4B78-8F0B-0862090DF17C}"/>
+    <hyperlink ref="E23" r:id="rId16" xr:uid="{4D2E9F39-BBF0-4ED5-A3F4-155FDCE0EE23}"/>
+    <hyperlink ref="E24" r:id="rId17" xr:uid="{2A107639-C50E-4692-BCD5-0196CE4739AB}"/>
     <hyperlink ref="E4" r:id="rId18" xr:uid="{844DA8A5-FB35-4F0B-A1F4-8116A748C40E}"/>
-    <hyperlink ref="E32" r:id="rId19" xr:uid="{5600F95F-40E7-4F55-A313-2023A5F400B9}"/>
-    <hyperlink ref="E33" r:id="rId20" xr:uid="{9D311E0B-996E-4B99-B32A-9F25E8B76079}"/>
-    <hyperlink ref="E31" r:id="rId21" xr:uid="{603F2D51-63FE-4820-93B9-30767E19C3CC}"/>
-    <hyperlink ref="E12" r:id="rId22" xr:uid="{28A0EBB7-2304-492C-A951-78F5F394482B}"/>
-    <hyperlink ref="E14" r:id="rId23" xr:uid="{6ED20A36-8F40-483A-BE25-4C87A2D92BFB}"/>
-    <hyperlink ref="E37" r:id="rId24" xr:uid="{658E5E28-83C4-44FC-A8A9-EE933E75693B}"/>
-    <hyperlink ref="E34" r:id="rId25" xr:uid="{6F005684-77F1-49B6-9BD6-CB4A7DAA5FC5}"/>
+    <hyperlink ref="E33" r:id="rId19" xr:uid="{5600F95F-40E7-4F55-A313-2023A5F400B9}"/>
+    <hyperlink ref="E34" r:id="rId20" xr:uid="{9D311E0B-996E-4B99-B32A-9F25E8B76079}"/>
+    <hyperlink ref="E32" r:id="rId21" xr:uid="{603F2D51-63FE-4820-93B9-30767E19C3CC}"/>
+    <hyperlink ref="E13" r:id="rId22" xr:uid="{28A0EBB7-2304-492C-A951-78F5F394482B}"/>
+    <hyperlink ref="E15" r:id="rId23" xr:uid="{6ED20A36-8F40-483A-BE25-4C87A2D92BFB}"/>
+    <hyperlink ref="E40" r:id="rId24" xr:uid="{658E5E28-83C4-44FC-A8A9-EE933E75693B}"/>
+    <hyperlink ref="E35" r:id="rId25" xr:uid="{6F005684-77F1-49B6-9BD6-CB4A7DAA5FC5}"/>
+    <hyperlink ref="E36" r:id="rId26" xr:uid="{E8969170-A8C2-4BE9-AF93-F1DA1981A4BD}"/>
+    <hyperlink ref="E37" r:id="rId27" xr:uid="{BE9117F2-C249-4F32-A092-D637A656EEA5}"/>
+    <hyperlink ref="E5" r:id="rId28" xr:uid="{028F87D3-6F53-4C03-8A9C-B168BA59CE8F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId26"/>
+  <legacyDrawing r:id="rId29"/>
 </worksheet>
 </file>
</xml_diff>